<commit_message>
Update csv, add csv 20260703_2
</commit_message>
<xml_diff>
--- a/TuVung/TuVung.xlsx
+++ b/TuVung/TuVung.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dxcportal-my.sharepoint.com/personal/dangtan_ngo2_dxc_com/Documents/studyingJapanese/TuVung/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="408" documentId="13_ncr:1_{AD9B2405-E9FD-4D4A-80B7-293F6A025480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10AE96A3-17C1-4782-AE6D-5CA8FA64F8EC}"/>
+  <xr:revisionPtr revIDLastSave="557" documentId="13_ncr:1_{AD9B2405-E9FD-4D4A-80B7-293F6A025480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E2763429-DCD6-4CCE-A670-E08B3994C5D1}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B0E4D7E1-AC8C-4A97-A943-EDCC3B3B5427}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1333" uniqueCount="1333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1407" uniqueCount="1407">
   <si>
     <t>機能</t>
   </si>
@@ -4662,6 +4662,247 @@
   </si>
   <si>
     <t>はかい - PHÁ HOẠI- phá hoại, phá hủy</t>
+  </si>
+  <si>
+    <t>層</t>
+  </si>
+  <si>
+    <t>そう - TẰNG- Đếm tầng, lớp : いっそう、にそう、さんそう</t>
+  </si>
+  <si>
+    <t>齟齬</t>
+  </si>
+  <si>
+    <t>そご - TRỞ NGỮ- sự mâu thuẫn,xung đột/ conflict</t>
+  </si>
+  <si>
+    <t>急務</t>
+  </si>
+  <si>
+    <t>きゅうむ - CẤP VỤ- Công việc khẩn cấp; nhiệm vụ cấp bách</t>
+  </si>
+  <si>
+    <t>途中</t>
+  </si>
+  <si>
+    <t>とちゅう - ĐỒ TRUNG- Dọc đường, Giữa chừng, Nửa đường</t>
+  </si>
+  <si>
+    <t>フィードバック</t>
+  </si>
+  <si>
+    <t>feedback - nhận xét</t>
+  </si>
+  <si>
+    <t>遅延</t>
+  </si>
+  <si>
+    <t>ちえん - TRÌ DUYÊN- trì hoãn</t>
+  </si>
+  <si>
+    <t>模擬</t>
+  </si>
+  <si>
+    <t>もぎ - MÔ NGHĨ- mô phỏng, bắt chước</t>
+  </si>
+  <si>
+    <t>避ける</t>
+  </si>
+  <si>
+    <t>よける - TỊ- ①さける Tránh né, trốn tránh ( trách nhiệm, mối nguy hiểm...)
+②よける　Phòng tránh ( côn trùng, bệnh...)</t>
+  </si>
+  <si>
+    <t>承認</t>
+  </si>
+  <si>
+    <t>しょうにん - THỪA NHẬN- sự xác nhận, phê duyệt</t>
+  </si>
+  <si>
+    <t>一環</t>
+  </si>
+  <si>
+    <t>いっかん - NHẤT HOÀN- 1 phần trong
+仕事の一環: một phần công việc.</t>
+  </si>
+  <si>
+    <t>真</t>
+  </si>
+  <si>
+    <t>まな - CHÂN- thật, thực tế
+真のURL:URL thật / URL thực tế / URL chính thức</t>
+  </si>
+  <si>
+    <t>同感</t>
+  </si>
+  <si>
+    <t>どうかん - ĐỒNG CẢM- Sự cùng ý kiến; sự cùng suy nghĩ
+同情：hán tự là đồng tình nhưng ý nghĩa là đồng cảm, cảm thương trước khó khăn của người khác
+同感：hán tự là đồng cảm nhưng ý nghĩa là đồng tình, cùng ý kiến với người khác</t>
+  </si>
+  <si>
+    <t>繋い</t>
+  </si>
+  <si>
+    <t>つなぐ - HỆ- Buộc vào; thắt; kết nối.
+インターネットを繋ぐkết nối internet</t>
+  </si>
+  <si>
+    <t>高負荷</t>
+  </si>
+  <si>
+    <t>こうふか - CAO PHỤ HÀ- Cường độ cao
+IT: 高負荷の処理: những xử lý nặng của máy tính.</t>
+  </si>
+  <si>
+    <t>並走</t>
+  </si>
+  <si>
+    <t>へいそう - TỊNH TẨU- Chạy song song</t>
+  </si>
+  <si>
+    <t>無限</t>
+  </si>
+  <si>
+    <t>むげん - VÔ HẠN- Sự vô hạn
+無限列車篇　chuyến tàu vô tận</t>
+  </si>
+  <si>
+    <t>過渡</t>
+  </si>
+  <si>
+    <t>かと - QUÁ ĐỘ- Giai đoạn chuyển tiếp (transition period) hoặc trạng thái quá độ</t>
+  </si>
+  <si>
+    <t>突合</t>
+  </si>
+  <si>
+    <t>つきあわせ - ĐỘT HỢP- matching: phù hợp.(member matching DB)</t>
+  </si>
+  <si>
+    <t>見落</t>
+  </si>
+  <si>
+    <t>みおとし - KIẾN LẠC- Nhìn sót, bỏ sót, không nhận thấy
+メッセージを見落としていました : Tôi đã bỏ sót tin nhắn</t>
+  </si>
+  <si>
+    <t>一歩一歩</t>
+  </si>
+  <si>
+    <t>いっぽいっぽ - NHẤT BỘ NHẤT BỘ- Từng bước. Step by step</t>
+  </si>
+  <si>
+    <t>スレッド</t>
+  </si>
+  <si>
+    <t>thread - chủ đề</t>
+  </si>
+  <si>
+    <t>共用</t>
+  </si>
+  <si>
+    <t>きょうよう - CỘNG DỤNG- Sự cùng nhau sử dụng; sự dùng chung;</t>
+  </si>
+  <si>
+    <t>素早く</t>
+  </si>
+  <si>
+    <t>すばやく - TỐ TẢO- Nhanh, nhanh chóng, Lẹ làng, lanh lợi</t>
+  </si>
+  <si>
+    <t>余裕</t>
+  </si>
+  <si>
+    <t>よゆう - DƯ DỤ- Dư thừa, rộng rãi,sớm hơn
+余裕を持って来るように。hãy cố gắng đến sớm hơn</t>
+  </si>
+  <si>
+    <t>順次</t>
+  </si>
+  <si>
+    <t>じゅんじ- THUẬN THỨ- Tuần tự, lần lượt
+Có mấy từ gần nghĩa với nhau là:
+順次、順番、逐次</t>
+  </si>
+  <si>
+    <t>丁寧</t>
+  </si>
+  <si>
+    <t>ていねい - ĐINH NINH- Sự lịch sự; sự cẩn thận.
+丁寧にありがとうございます。</t>
+  </si>
+  <si>
+    <t>十分</t>
+  </si>
+  <si>
+    <t>じゅうぶん - THẬP PHÂN- Đầy đủ; hoàn toàn; chặt chẽ; sít sao; rõ</t>
+  </si>
+  <si>
+    <t>軽微</t>
+  </si>
+  <si>
+    <t>けいび - KHINH VI- không đáng kể, nhỏ</t>
+  </si>
+  <si>
+    <t>迅速</t>
+  </si>
+  <si>
+    <t>じんそく - TẤN TỐC- Sự mau lẹ; sự nhanh chóng.
+迅速なご対応助かりました。</t>
+  </si>
+  <si>
+    <t>コロコロ</t>
+  </si>
+  <si>
+    <t>xoành xoạch
+コロコロ変化する: thay đổi xoành xoạch</t>
+  </si>
+  <si>
+    <t>協力</t>
+  </si>
+  <si>
+    <t>きょうりょく - HIỆP LỰC- Sự hợp tác; hợp tác; sự hiệp lực; hiệp lực
+1。能力(のうりょく)năng lực
+2。努力(どりょく)nỗ lực
+3。協力(きょうりょく)chung sức, hợp tác , hiệp lực</t>
+  </si>
+  <si>
+    <t>一部</t>
+  </si>
+  <si>
+    <t>いちぶ - NHẤT BỘ- Một phần</t>
+  </si>
+  <si>
+    <t>混乱</t>
+  </si>
+  <si>
+    <t>こんらん - HỖN LOẠN- Lúng túng; hỗn loạn</t>
+  </si>
+  <si>
+    <t>大量</t>
+  </si>
+  <si>
+    <t>たいりょう - ĐẠI LƯỢNG- Số lượng lớn</t>
+  </si>
+  <si>
+    <t>増強</t>
+  </si>
+  <si>
+    <t>ぞうきょう - TĂNG CƯỜNG- Tăng cường củng cố</t>
+  </si>
+  <si>
+    <t>賄う</t>
+  </si>
+  <si>
+    <t>まかなう - HỐI- Nghĩa 1: trang trải, chi trả, ...
+Nghĩa 2: cung cấp</t>
+  </si>
+  <si>
+    <t>段階</t>
+  </si>
+  <si>
+    <t>きだはし - ĐOẠN GIAI- các bước, giai đoạn</t>
   </si>
 </sst>
 </file>
@@ -5140,7 +5381,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{572AC1B0-BE23-45AF-BF40-510643C6C658}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:B705"/>
+  <dimension ref="A1:B742"/>
   <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="18.5546875" style="2" bestFit="1" customWidth="1"/>
@@ -10554,6 +10795,302 @@
       </c>
       <c r="B705" s="1" t="s">
         <v>1332</v>
+      </c>
+    </row>
+    <row r="706" spans="1:2" ht="31.5">
+      <c r="A706" s="11" t="s">
+        <v>1333</v>
+      </c>
+      <c r="B706" s="1" t="s">
+        <v>1334</v>
+      </c>
+    </row>
+    <row r="707" spans="1:2" ht="31.5">
+      <c r="A707" s="2" t="s">
+        <v>1335</v>
+      </c>
+      <c r="B707" s="1" t="s">
+        <v>1336</v>
+      </c>
+    </row>
+    <row r="708" spans="1:2" ht="31.5">
+      <c r="A708" s="2" t="s">
+        <v>1337</v>
+      </c>
+      <c r="B708" s="1" t="s">
+        <v>1338</v>
+      </c>
+    </row>
+    <row r="709" spans="1:2" ht="31.5">
+      <c r="A709" s="2" t="s">
+        <v>1339</v>
+      </c>
+      <c r="B709" s="1" t="s">
+        <v>1340</v>
+      </c>
+    </row>
+    <row r="710" spans="1:2">
+      <c r="A710" s="2" t="s">
+        <v>1341</v>
+      </c>
+      <c r="B710" s="1" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="711" spans="1:2">
+      <c r="A711" s="2" t="s">
+        <v>1343</v>
+      </c>
+      <c r="B711" s="1" t="s">
+        <v>1344</v>
+      </c>
+    </row>
+    <row r="712" spans="1:2">
+      <c r="A712" s="2" t="s">
+        <v>1345</v>
+      </c>
+      <c r="B712" s="1" t="s">
+        <v>1346</v>
+      </c>
+    </row>
+    <row r="713" spans="1:2" ht="63">
+      <c r="A713" s="2" t="s">
+        <v>1347</v>
+      </c>
+      <c r="B713" s="1" t="s">
+        <v>1348</v>
+      </c>
+    </row>
+    <row r="714" spans="1:2" ht="31.5">
+      <c r="A714" s="2" t="s">
+        <v>1349</v>
+      </c>
+      <c r="B714" s="1" t="s">
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="715" spans="1:2" ht="31.5">
+      <c r="A715" s="2" t="s">
+        <v>1351</v>
+      </c>
+      <c r="B715" s="1" t="s">
+        <v>1352</v>
+      </c>
+    </row>
+    <row r="716" spans="1:2" ht="47.25">
+      <c r="A716" s="2" t="s">
+        <v>1353</v>
+      </c>
+      <c r="B716" s="1" t="s">
+        <v>1354</v>
+      </c>
+    </row>
+    <row r="717" spans="1:2" ht="126">
+      <c r="A717" s="2" t="s">
+        <v>1355</v>
+      </c>
+      <c r="B717" s="1" t="s">
+        <v>1356</v>
+      </c>
+    </row>
+    <row r="718" spans="1:2" ht="31.5">
+      <c r="A718" s="2" t="s">
+        <v>1357</v>
+      </c>
+      <c r="B718" s="1" t="s">
+        <v>1358</v>
+      </c>
+    </row>
+    <row r="719" spans="1:2" ht="47.25">
+      <c r="A719" s="2" t="s">
+        <v>1359</v>
+      </c>
+      <c r="B719" s="1" t="s">
+        <v>1360</v>
+      </c>
+    </row>
+    <row r="720" spans="1:2">
+      <c r="A720" s="2" t="s">
+        <v>1361</v>
+      </c>
+      <c r="B720" s="1" t="s">
+        <v>1362</v>
+      </c>
+    </row>
+    <row r="721" spans="1:2" ht="31.5">
+      <c r="A721" s="2" t="s">
+        <v>1363</v>
+      </c>
+      <c r="B721" s="1" t="s">
+        <v>1364</v>
+      </c>
+    </row>
+    <row r="722" spans="1:2" ht="47.25">
+      <c r="A722" s="2" t="s">
+        <v>1365</v>
+      </c>
+      <c r="B722" s="1" t="s">
+        <v>1366</v>
+      </c>
+    </row>
+    <row r="723" spans="1:2" ht="31.5">
+      <c r="A723" s="2" t="s">
+        <v>1367</v>
+      </c>
+      <c r="B723" s="1" t="s">
+        <v>1368</v>
+      </c>
+    </row>
+    <row r="724" spans="1:2" ht="63">
+      <c r="A724" s="2" t="s">
+        <v>1369</v>
+      </c>
+      <c r="B724" s="1" t="s">
+        <v>1370</v>
+      </c>
+    </row>
+    <row r="725" spans="1:2" ht="31.5">
+      <c r="A725" s="2" t="s">
+        <v>1371</v>
+      </c>
+      <c r="B725" s="1" t="s">
+        <v>1372</v>
+      </c>
+    </row>
+    <row r="726" spans="1:2">
+      <c r="A726" s="2" t="s">
+        <v>1373</v>
+      </c>
+      <c r="B726" s="1" t="s">
+        <v>1374</v>
+      </c>
+    </row>
+    <row r="727" spans="1:2" ht="31.5">
+      <c r="A727" s="2" t="s">
+        <v>1375</v>
+      </c>
+      <c r="B727" s="1" t="s">
+        <v>1376</v>
+      </c>
+    </row>
+    <row r="728" spans="1:2" ht="31.5">
+      <c r="A728" s="2" t="s">
+        <v>1377</v>
+      </c>
+      <c r="B728" s="1" t="s">
+        <v>1378</v>
+      </c>
+    </row>
+    <row r="729" spans="1:2" ht="63">
+      <c r="A729" s="2" t="s">
+        <v>1379</v>
+      </c>
+      <c r="B729" s="1" t="s">
+        <v>1380</v>
+      </c>
+    </row>
+    <row r="730" spans="1:2" ht="47.25">
+      <c r="A730" s="2" t="s">
+        <v>1381</v>
+      </c>
+      <c r="B730" s="1" t="s">
+        <v>1382</v>
+      </c>
+    </row>
+    <row r="731" spans="1:2" ht="47.25">
+      <c r="A731" s="2" t="s">
+        <v>1383</v>
+      </c>
+      <c r="B731" s="1" t="s">
+        <v>1384</v>
+      </c>
+    </row>
+    <row r="732" spans="1:2" ht="31.5">
+      <c r="A732" s="2" t="s">
+        <v>1385</v>
+      </c>
+      <c r="B732" s="1" t="s">
+        <v>1386</v>
+      </c>
+    </row>
+    <row r="733" spans="1:2">
+      <c r="A733" s="2" t="s">
+        <v>1387</v>
+      </c>
+      <c r="B733" s="1" t="s">
+        <v>1388</v>
+      </c>
+    </row>
+    <row r="734" spans="1:2" ht="47.25">
+      <c r="A734" s="2" t="s">
+        <v>1389</v>
+      </c>
+      <c r="B734" s="1" t="s">
+        <v>1390</v>
+      </c>
+    </row>
+    <row r="735" spans="1:2" ht="31.5">
+      <c r="A735" s="2" t="s">
+        <v>1391</v>
+      </c>
+      <c r="B735" s="1" t="s">
+        <v>1392</v>
+      </c>
+    </row>
+    <row r="736" spans="1:2" ht="94.5">
+      <c r="A736" s="2" t="s">
+        <v>1393</v>
+      </c>
+      <c r="B736" s="1" t="s">
+        <v>1394</v>
+      </c>
+    </row>
+    <row r="737" spans="1:2">
+      <c r="A737" s="2" t="s">
+        <v>1395</v>
+      </c>
+      <c r="B737" s="1" t="s">
+        <v>1396</v>
+      </c>
+    </row>
+    <row r="738" spans="1:2" ht="31.5">
+      <c r="A738" s="2" t="s">
+        <v>1397</v>
+      </c>
+      <c r="B738" s="1" t="s">
+        <v>1398</v>
+      </c>
+    </row>
+    <row r="739" spans="1:2">
+      <c r="A739" s="2" t="s">
+        <v>1399</v>
+      </c>
+      <c r="B739" s="1" t="s">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="740" spans="1:2" ht="31.5">
+      <c r="A740" s="2" t="s">
+        <v>1401</v>
+      </c>
+      <c r="B740" s="1" t="s">
+        <v>1402</v>
+      </c>
+    </row>
+    <row r="741" spans="1:2" ht="47.25">
+      <c r="A741" s="2" t="s">
+        <v>1403</v>
+      </c>
+      <c r="B741" s="1" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="742" spans="1:2" ht="31.5">
+      <c r="A742" s="2" t="s">
+        <v>1405</v>
+      </c>
+      <c r="B742" s="1" t="s">
+        <v>1406</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add N2 and vocabulary CSV files
</commit_message>
<xml_diff>
--- a/TuVung/TuVung.xlsx
+++ b/TuVung/TuVung.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dxcportal-my.sharepoint.com/personal/dangtan_ngo2_dxc_com/Documents/studyingJapanese/TuVung/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="683" documentId="13_ncr:1_{AD9B2405-E9FD-4D4A-80B7-293F6A025480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{43FD95E8-C2B5-463E-A13C-5747813B7433}"/>
+  <xr:revisionPtr revIDLastSave="839" documentId="13_ncr:1_{AD9B2405-E9FD-4D4A-80B7-293F6A025480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8156ADC7-B663-4244-8E6B-96DDF066E7CE}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B0E4D7E1-AC8C-4A97-A943-EDCC3B3B5427}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1495" uniqueCount="1495">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1593" uniqueCount="1593">
   <si>
     <t>機能</t>
   </si>
@@ -5179,6 +5179,356 @@
   </si>
   <si>
     <t>きんゆうきかん - KIM DUNG KI QUAN- Tổ chức tín dụng, tổ chức tài chính</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+契約割販</t>
+  </si>
+  <si>
+    <t>けいやくかっぱん ( Khế Ước Cát Phiến) Hợp đồng trả góp</t>
+  </si>
+  <si>
+    <t>読み込み</t>
+  </si>
+  <si>
+    <t>よみこみ - ĐỘC NHẬP - Load / đọc, tải
+読み込み中: loading</t>
+  </si>
+  <si>
+    <t>過程</t>
+  </si>
+  <si>
+    <t>かてい - QUÁ TRÌNH- Quá trình; giai đoạn
+Phân biệt giữa 過程　経過
+過程 : Quá trình, là một bước trong một chuỗi những thay đổi. 生産過程 : quá trình sinh sản
+経過 : Tiến trình, ko chỉ là một bước đơn thuần, nó là cả một loạt những thay đổi dần dần.</t>
+  </si>
+  <si>
+    <t>浄化</t>
+  </si>
+  <si>
+    <t>じょうか - TỊNH HÓA- Làm sạch, thanh tẩy
+浄化データ = dữ liệu đã xóa/che thông tin nhạy cảm (PAN, thẻ, PII...)</t>
+  </si>
+  <si>
+    <t>為</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ため - VI - Bởi vì; mục đích là; Để
+本会員顧客をユニークにする為のID
+ID dùng để phân biệt duy nhất một khách hàng hội viên chính.
+</t>
+  </si>
+  <si>
+    <t>売上受入</t>
+  </si>
+  <si>
+    <t xml:space="preserve">うりあげ うけいれ - MẠI THƯỢNG THỤ NHẬP-nhận doanh thu
+=&gt; 売上受入 = quá trình tiếp nhận dữ liệu giao dịch bán hàng vào hệ thống.  </t>
+  </si>
+  <si>
+    <t>払戻し</t>
+  </si>
+  <si>
+    <t>はらいもどし- PHẤT LỆ - hoàn tiền, hoàn trả, refund.</t>
+  </si>
+  <si>
+    <t>誤打</t>
+  </si>
+  <si>
+    <t>ごだ - NGỘ ĐẢ - nhập sai thao tác / nhập nhầm dữ liệu</t>
+  </si>
+  <si>
+    <t>精算</t>
+  </si>
+  <si>
+    <t>せいさん - TINH TOÁN- Đối soát và thanh quyết toán cuối cùng
+精算先加盟店番号: Mã định danh của merchant nhận tiền thanh quyết toán.</t>
+  </si>
+  <si>
+    <t>精算先加盟店番号</t>
+  </si>
+  <si>
+    <t xml:space="preserve">せいさんさき かめいてん ばんごう -TINH TOÁN TIÊN GIA MINH ĐIẾM PHIÊN HÀO - Mã số merchant nhận thanh quyết toán
+加盟店  - Merchant </t>
+  </si>
+  <si>
+    <t>示す</t>
+  </si>
+  <si>
+    <t xml:space="preserve">しめす - KÌ- Biểu hiện ra; chỉ ra; cho thấy/express </t>
+  </si>
+  <si>
+    <t>優待</t>
+  </si>
+  <si>
+    <t>ゆうたい - ƯU ĐÃI- Ưu đãi.</t>
+  </si>
+  <si>
+    <t>累積</t>
+  </si>
+  <si>
+    <t>るいせき - LUY TÍCH- Tích lũy, cộng dồn, lũy kế
+ポイントを累積する期間の月数を設定する。
+→ Thiết lập số tháng của kỳ tích lũy điểm</t>
+  </si>
+  <si>
+    <t>締日</t>
+  </si>
+  <si>
+    <t>しめび - Đế Nhật - ngày chốt</t>
+  </si>
+  <si>
+    <t>累計</t>
+  </si>
+  <si>
+    <t>るいけい - LUY KẾ- Lũy kế; tích luỹ
+累計ポイント điểm tích luỹ</t>
+  </si>
+  <si>
+    <t>マイナス</t>
+  </si>
+  <si>
+    <t>Minus (-), âm, giảm trừ, số âm
+当期度交換可能ポイントがマイナスの場合
+→ Trường hợp điểm có thể đổi trong kỳ hiện tại bị âm.</t>
+  </si>
+  <si>
+    <t>相殺</t>
+  </si>
+  <si>
+    <t>そうさつ - TƯƠNG SÁT- Bù trừ, cấn trừ, offset
+相殺処理 (xử lý bù trừ)</t>
+  </si>
+  <si>
+    <t>債権</t>
+  </si>
+  <si>
+    <t>さいけん - TRÁI QUYỀN- Khoản phải thu, quyền đòi nợ, credit receivable
+カード会社 → 債権者 (chủ nợ)
+会員顧客 → 債務者 (người phải trả nợ)</t>
+  </si>
+  <si>
+    <t>採番</t>
+  </si>
+  <si>
+    <t>さいばん - THẢI PHIÊN- Đánh số, cấp số, gán số định danh tự động
+ポイント種別IDで採番
+→ Sinh số dựa trên Point Type ID</t>
+  </si>
+  <si>
+    <t>グレード</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Grade / Hạng / Cấp bậc
+グレード付与有無フラグ
+→ Cờ xác định có áp dụng cơ chế hạng thành viên hay không.</t>
+  </si>
+  <si>
+    <t>引換</t>
+  </si>
+  <si>
+    <t>ひきかえ - DẪN HOÁN- Đổi lấy, quy đổi, đổi thưởng (redeem/exchange)
+ポイント引換商品管理
+→ Quản lý sản phẩm đổi thưởng.</t>
+  </si>
+  <si>
+    <t>提携</t>
+  </si>
+  <si>
+    <t>ていけい - ĐỀ HUỀ- liên kết, hợp tác
+提携ATM: máy rút tiền có liên kết (rút được tiền ngân hàng không cùng hệ thống)</t>
+  </si>
+  <si>
+    <t>繰越</t>
+  </si>
+  <si>
+    <t>くりこし - SÀO VIỆT-Chuyển sang kỳ sau, carry forward, carry over
+前月繰越金
+Tiền từ tháng trước chuyển sang</t>
+  </si>
+  <si>
+    <t>切替</t>
+  </si>
+  <si>
+    <t>きりかえ - THIẾT THẾ- Chuyển đổi, thay đổi, switch</t>
+  </si>
+  <si>
+    <t>階層</t>
+  </si>
+  <si>
+    <t>かいそう - GIAI TẰNG- Giai tầng; tầng lớp,hierarchy (engineer field), layer</t>
+  </si>
+  <si>
+    <t>細分</t>
+  </si>
+  <si>
+    <t>さいぶん - TẾ PHÂN- Phân nhỏ, chia nhỏ, phân chia chi tiết hơn
+顧客区分を細分する
+→ Phân chia chi tiết hơn các nhóm khách hàng.</t>
+  </si>
+  <si>
+    <t>導出</t>
+  </si>
+  <si>
+    <t>どうしゅつ - ĐẠO XUẤT- Suy ra, tính toán để tạo ra giá trị, derive
+CASE
+ WHEN ...
+ THEN ...
+ ELSE ...
+END
+→ Logic này gọi là 導出ロジック.</t>
+  </si>
+  <si>
+    <t>形態</t>
+  </si>
+  <si>
+    <t>けいたい - HÌNH THÁI- Hình thái; hình thức; dạng; loại hình</t>
+  </si>
+  <si>
+    <t>完済</t>
+  </si>
+  <si>
+    <t>かんさい - HOÀN TẾ- Trả hết nợ, thanh toán toàn bộ dư nợ, Paid off in full</t>
+  </si>
+  <si>
+    <t>遅損金</t>
+  </si>
+  <si>
+    <t>ちそんきん - TRÌ TỔN KIM- khoản tiền phát sinh do khách hàng thanh toán chậm so với thời hạn quy định.</t>
+  </si>
+  <si>
+    <t>元金</t>
+  </si>
+  <si>
+    <t>もときん - NGUYÊN KIM- Tiền vốn; tiền vốn</t>
+  </si>
+  <si>
+    <t>利息</t>
+  </si>
+  <si>
+    <t>りそく - LỢI TỨC- ố tiền lãi thu dc khi đầu tư, gửi ngân hàng ( Đồng/USD/yên)
+金利：lãi xuất bên vay trả ( đơn vị % )
+利子: tiền lãi bên vay trả ( đơn vị Đồng/ yên/ USD)
+VD vay 100万円（元本）×0.03％（金利）=3万円 (利子）
+利回り :　lợi tức/ cổ tức ( khi bạn đầu tư/ gửi ngân hàng thu lời dc % )</t>
+  </si>
+  <si>
+    <t>和暦</t>
+  </si>
+  <si>
+    <t>われき - HÒA LỊCH- Lịch Nhật Bản theo niên hiệu Thiên hoàng (Japanese Era Calendar)</t>
+  </si>
+  <si>
+    <t>外信</t>
+  </si>
+  <si>
+    <t>がいしん - NGOẠI TÍN- Tin tức từ nước ngoài, điện tín/thông tin từ nước ngoài, foreign news dispatch</t>
+  </si>
+  <si>
+    <t>姓</t>
+  </si>
+  <si>
+    <t>かばね - TÍNH- =名字: họ</t>
+  </si>
+  <si>
+    <t>公的</t>
+  </si>
+  <si>
+    <t>こうてき - CÔNG ĐÍCH- Công, chính thức, thuộc cơ quan nhà nước hoặc tổ chức công quyền
+公的機関
+→ Cơ quan công quyền / cơ quan nhà nước.
+公的書類
+→ Giấy tờ chính thức do cơ quan nhà nước cấp.</t>
+  </si>
+  <si>
+    <t>昭和</t>
+  </si>
+  <si>
+    <t>しょうわ  -CHIÊU HÒA- Thời đại Chiêu Hòa 1926–1989</t>
+  </si>
+  <si>
+    <t>リボ使用</t>
+  </si>
+  <si>
+    <t>りぼしよう - Sử dụng hình thức thanh toán Revolving (Revolving Payment)
+hay thường gọi là trả góp vòng quay (リボ払い).
+リボ là gì?
+リボ = リボルビング払い (Revolving Payment)
+Khách hàng không trả toàn bộ dư nợ thẻ mỗi tháng mà trả một khoản cố định hàng tháng.</t>
+  </si>
+  <si>
+    <t>ﾏﾝｽﾘｰｸﾘｱ</t>
+  </si>
+  <si>
+    <t>Monthly Clear -Thanh toán toàn bộ dư nợ phát sinh trong tháng vào kỳ thanh toán tiếp theo.</t>
+  </si>
+  <si>
+    <t>元本</t>
+  </si>
+  <si>
+    <t>げんぽん - NGUYÊN BỔN- Tiền gốc, Vốn gốc ban đầu khi cho vay</t>
+  </si>
+  <si>
+    <t>督促</t>
+  </si>
+  <si>
+    <t>とくそく - ĐỐC XÚC- Sự đốc thúc; sự thúc giục</t>
+  </si>
+  <si>
+    <t>未納</t>
+  </si>
+  <si>
+    <t>みのう - VỊ NẠP- Sự vỡ nợ; sự quá hạn thanh toán; sự chưa thanh toán.</t>
+  </si>
+  <si>
+    <t>返戻</t>
+  </si>
+  <si>
+    <t>へんれい - PHẢN LỆ- Sự trả lại, sự gửi lại, hoàn trả
+借用した本を返戻する。hoàn trả sách đã mượn</t>
+  </si>
+  <si>
+    <t>償却</t>
+  </si>
+  <si>
+    <t>しょうきゃく - THƯỜNG KHƯỚC- Khấu hao ,khấu trừ</t>
+  </si>
+  <si>
+    <t>徴収</t>
+  </si>
+  <si>
+    <t>ちょうしゅう - TRƯNG THU- Thu (thuế, tiền)</t>
+  </si>
+  <si>
+    <t>配偶</t>
+  </si>
+  <si>
+    <t>はいぐう - PHỐI NGẪU- Sự phối ngẫu ( vợ/chồng)
+配偶者：NGƯỜI PHỐI NGẪU( VỢ/CHỒNG)</t>
+  </si>
+  <si>
+    <t>人為</t>
+  </si>
+  <si>
+    <t>じんい - NHÂN VI- yếu tố xuất phát từ hành động của con ngườ</t>
+  </si>
+  <si>
+    <t>フリー入力</t>
+  </si>
+  <si>
+    <t>Free Input - Nhập tự do, nhập thủ công, không bị giới hạn bởi danh sách chọn hoặc code master
+フリー入力可
+→ Cho phép nhập tự do.
+フリー入力項目
+→ Trường nhập tự do.</t>
+  </si>
+  <si>
+    <t>否か</t>
+  </si>
+  <si>
+    <t>いなか - PHỦ- phủ định (của một Danh từ, Tính từ, Động từ nào đó). 
+VD: 美味しいか否か: ngon hay không ngon. 出席するか否か: có mặt hay không có mặt.</t>
   </si>
 </sst>
 </file>
@@ -5274,7 +5624,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -5291,6 +5641,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5657,7 +6010,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{572AC1B0-BE23-45AF-BF40-510643C6C658}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:B786"/>
+  <dimension ref="A1:B835"/>
   <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="18.5546875" style="2" bestFit="1" customWidth="1"/>
@@ -7984,7 +8337,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="291" spans="1:2" ht="94.5">
+    <row r="291" spans="1:2" ht="78.75">
       <c r="A291" s="2" t="s">
         <v>582</v>
       </c>
@@ -9241,7 +9594,7 @@
         <v>876</v>
       </c>
     </row>
-    <row r="477" spans="1:2" ht="126">
+    <row r="477" spans="1:2" ht="141.75">
       <c r="A477" s="2" t="s">
         <v>877</v>
       </c>
@@ -9449,7 +9802,7 @@
         <v>927</v>
       </c>
     </row>
-    <row r="503" spans="1:2" ht="78.75">
+    <row r="503" spans="1:2" ht="94.5">
       <c r="A503" s="2" t="s">
         <v>928</v>
       </c>
@@ -11719,6 +12072,398 @@
       </c>
       <c r="B786" s="1" t="s">
         <v>1494</v>
+      </c>
+    </row>
+    <row r="787" spans="1:2" ht="31.5">
+      <c r="A787" s="12" t="s">
+        <v>1495</v>
+      </c>
+      <c r="B787" s="1" t="s">
+        <v>1496</v>
+      </c>
+    </row>
+    <row r="788" spans="1:2" ht="31.5">
+      <c r="A788" s="2" t="s">
+        <v>1497</v>
+      </c>
+      <c r="B788" s="1" t="s">
+        <v>1498</v>
+      </c>
+    </row>
+    <row r="789" spans="1:2" ht="141.75">
+      <c r="A789" s="2" t="s">
+        <v>1499</v>
+      </c>
+      <c r="B789" s="1" t="s">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="790" spans="1:2" ht="63">
+      <c r="A790" s="2" t="s">
+        <v>1501</v>
+      </c>
+      <c r="B790" s="1" t="s">
+        <v>1502</v>
+      </c>
+    </row>
+    <row r="791" spans="1:2" ht="78.75">
+      <c r="A791" s="2" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B791" s="1" t="s">
+        <v>1504</v>
+      </c>
+    </row>
+    <row r="792" spans="1:2" ht="63">
+      <c r="A792" s="2" t="s">
+        <v>1505</v>
+      </c>
+      <c r="B792" s="1" t="s">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="793" spans="1:2" ht="31.5">
+      <c r="A793" s="2" t="s">
+        <v>1507</v>
+      </c>
+      <c r="B793" s="1" t="s">
+        <v>1508</v>
+      </c>
+    </row>
+    <row r="794" spans="1:2" ht="31.5">
+      <c r="A794" s="2" t="s">
+        <v>1509</v>
+      </c>
+      <c r="B794" s="1" t="s">
+        <v>1510</v>
+      </c>
+    </row>
+    <row r="795" spans="1:2" ht="63">
+      <c r="A795" s="2" t="s">
+        <v>1511</v>
+      </c>
+      <c r="B795" s="1" t="s">
+        <v>1512</v>
+      </c>
+    </row>
+    <row r="796" spans="1:2" ht="78.75">
+      <c r="A796" s="2" t="s">
+        <v>1513</v>
+      </c>
+      <c r="B796" s="1" t="s">
+        <v>1514</v>
+      </c>
+    </row>
+    <row r="797" spans="1:2" ht="31.5">
+      <c r="A797" s="2" t="s">
+        <v>1515</v>
+      </c>
+      <c r="B797" s="1" t="s">
+        <v>1516</v>
+      </c>
+    </row>
+    <row r="798" spans="1:2">
+      <c r="A798" s="2" t="s">
+        <v>1517</v>
+      </c>
+      <c r="B798" s="1" t="s">
+        <v>1518</v>
+      </c>
+    </row>
+    <row r="799" spans="1:2" ht="78.75">
+      <c r="A799" s="2" t="s">
+        <v>1519</v>
+      </c>
+      <c r="B799" s="1" t="s">
+        <v>1520</v>
+      </c>
+    </row>
+    <row r="800" spans="1:2">
+      <c r="A800" s="2" t="s">
+        <v>1521</v>
+      </c>
+      <c r="B800" s="1" t="s">
+        <v>1522</v>
+      </c>
+    </row>
+    <row r="801" spans="1:2" ht="31.5">
+      <c r="A801" s="2" t="s">
+        <v>1523</v>
+      </c>
+      <c r="B801" s="1" t="s">
+        <v>1524</v>
+      </c>
+    </row>
+    <row r="802" spans="1:2" ht="63">
+      <c r="A802" s="2" t="s">
+        <v>1525</v>
+      </c>
+      <c r="B802" s="1" t="s">
+        <v>1526</v>
+      </c>
+    </row>
+    <row r="803" spans="1:2" ht="47.25">
+      <c r="A803" s="2" t="s">
+        <v>1527</v>
+      </c>
+      <c r="B803" s="1" t="s">
+        <v>1528</v>
+      </c>
+    </row>
+    <row r="804" spans="1:2" ht="63">
+      <c r="A804" s="2" t="s">
+        <v>1529</v>
+      </c>
+      <c r="B804" s="1" t="s">
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="805" spans="1:2" ht="63">
+      <c r="A805" s="2" t="s">
+        <v>1531</v>
+      </c>
+      <c r="B805" s="1" t="s">
+        <v>1532</v>
+      </c>
+    </row>
+    <row r="806" spans="1:2" ht="63">
+      <c r="A806" s="2" t="s">
+        <v>1533</v>
+      </c>
+      <c r="B806" s="1" t="s">
+        <v>1534</v>
+      </c>
+    </row>
+    <row r="807" spans="1:2" ht="63">
+      <c r="A807" s="2" t="s">
+        <v>1535</v>
+      </c>
+      <c r="B807" s="1" t="s">
+        <v>1536</v>
+      </c>
+    </row>
+    <row r="808" spans="1:2" ht="63">
+      <c r="A808" s="2" t="s">
+        <v>1537</v>
+      </c>
+      <c r="B808" s="1" t="s">
+        <v>1538</v>
+      </c>
+    </row>
+    <row r="809" spans="1:2" ht="63">
+      <c r="A809" s="2" t="s">
+        <v>1539</v>
+      </c>
+      <c r="B809" s="1" t="s">
+        <v>1540</v>
+      </c>
+    </row>
+    <row r="810" spans="1:2" ht="31.5">
+      <c r="A810" s="2" t="s">
+        <v>1541</v>
+      </c>
+      <c r="B810" s="1" t="s">
+        <v>1542</v>
+      </c>
+    </row>
+    <row r="811" spans="1:2" ht="31.5">
+      <c r="A811" s="2" t="s">
+        <v>1543</v>
+      </c>
+      <c r="B811" s="1" t="s">
+        <v>1544</v>
+      </c>
+    </row>
+    <row r="812" spans="1:2" ht="78.75">
+      <c r="A812" s="2" t="s">
+        <v>1545</v>
+      </c>
+      <c r="B812" s="1" t="s">
+        <v>1546</v>
+      </c>
+    </row>
+    <row r="813" spans="1:2" ht="126">
+      <c r="A813" s="2" t="s">
+        <v>1547</v>
+      </c>
+      <c r="B813" s="1" t="s">
+        <v>1548</v>
+      </c>
+    </row>
+    <row r="814" spans="1:2" ht="31.5">
+      <c r="A814" s="11" t="s">
+        <v>1549</v>
+      </c>
+      <c r="B814" s="1" t="s">
+        <v>1550</v>
+      </c>
+    </row>
+    <row r="815" spans="1:2" ht="31.5">
+      <c r="A815" s="2" t="s">
+        <v>1551</v>
+      </c>
+      <c r="B815" s="1" t="s">
+        <v>1552</v>
+      </c>
+    </row>
+    <row r="816" spans="1:2" ht="47.25">
+      <c r="A816" s="2" t="s">
+        <v>1553</v>
+      </c>
+      <c r="B816" s="1" t="s">
+        <v>1554</v>
+      </c>
+    </row>
+    <row r="817" spans="1:2" ht="31.5">
+      <c r="A817" s="2" t="s">
+        <v>1555</v>
+      </c>
+      <c r="B817" s="1" t="s">
+        <v>1556</v>
+      </c>
+    </row>
+    <row r="818" spans="1:2" ht="173.25">
+      <c r="A818" s="2" t="s">
+        <v>1557</v>
+      </c>
+      <c r="B818" s="1" t="s">
+        <v>1558</v>
+      </c>
+    </row>
+    <row r="819" spans="1:2" ht="47.25">
+      <c r="A819" s="2" t="s">
+        <v>1559</v>
+      </c>
+      <c r="B819" s="1" t="s">
+        <v>1560</v>
+      </c>
+    </row>
+    <row r="820" spans="1:2" ht="47.25">
+      <c r="A820" s="2" t="s">
+        <v>1561</v>
+      </c>
+      <c r="B820" s="1" t="s">
+        <v>1562</v>
+      </c>
+    </row>
+    <row r="821" spans="1:2">
+      <c r="A821" s="2" t="s">
+        <v>1563</v>
+      </c>
+      <c r="B821" s="1" t="s">
+        <v>1564</v>
+      </c>
+    </row>
+    <row r="822" spans="1:2" ht="141.75">
+      <c r="A822" s="2" t="s">
+        <v>1565</v>
+      </c>
+      <c r="B822" s="1" t="s">
+        <v>1566</v>
+      </c>
+    </row>
+    <row r="823" spans="1:2" ht="31.5">
+      <c r="A823" s="2" t="s">
+        <v>1567</v>
+      </c>
+      <c r="B823" s="1" t="s">
+        <v>1568</v>
+      </c>
+    </row>
+    <row r="824" spans="1:2" ht="157.5">
+      <c r="A824" s="2" t="s">
+        <v>1569</v>
+      </c>
+      <c r="B824" s="1" t="s">
+        <v>1570</v>
+      </c>
+    </row>
+    <row r="825" spans="1:2" ht="47.25">
+      <c r="A825" s="2" t="s">
+        <v>1571</v>
+      </c>
+      <c r="B825" s="1" t="s">
+        <v>1572</v>
+      </c>
+    </row>
+    <row r="826" spans="1:2" ht="31.5">
+      <c r="A826" s="2" t="s">
+        <v>1573</v>
+      </c>
+      <c r="B826" s="1" t="s">
+        <v>1574</v>
+      </c>
+    </row>
+    <row r="827" spans="1:2" ht="31.5">
+      <c r="A827" s="2" t="s">
+        <v>1575</v>
+      </c>
+      <c r="B827" s="1" t="s">
+        <v>1576</v>
+      </c>
+    </row>
+    <row r="828" spans="1:2" ht="31.5">
+      <c r="A828" s="2" t="s">
+        <v>1577</v>
+      </c>
+      <c r="B828" s="1" t="s">
+        <v>1578</v>
+      </c>
+    </row>
+    <row r="829" spans="1:2" ht="63">
+      <c r="A829" s="2" t="s">
+        <v>1579</v>
+      </c>
+      <c r="B829" s="1" t="s">
+        <v>1580</v>
+      </c>
+    </row>
+    <row r="830" spans="1:2" ht="31.5">
+      <c r="A830" s="2" t="s">
+        <v>1581</v>
+      </c>
+      <c r="B830" s="1" t="s">
+        <v>1582</v>
+      </c>
+    </row>
+    <row r="831" spans="1:2" ht="31.5">
+      <c r="A831" s="2" t="s">
+        <v>1583</v>
+      </c>
+      <c r="B831" s="1" t="s">
+        <v>1584</v>
+      </c>
+    </row>
+    <row r="832" spans="1:2" ht="63">
+      <c r="A832" s="2" t="s">
+        <v>1585</v>
+      </c>
+      <c r="B832" s="1" t="s">
+        <v>1586</v>
+      </c>
+    </row>
+    <row r="833" spans="1:2" ht="31.5">
+      <c r="A833" s="2" t="s">
+        <v>1587</v>
+      </c>
+      <c r="B833" s="1" t="s">
+        <v>1588</v>
+      </c>
+    </row>
+    <row r="834" spans="1:2" ht="110.25">
+      <c r="A834" s="2" t="s">
+        <v>1589</v>
+      </c>
+      <c r="B834" s="1" t="s">
+        <v>1590</v>
+      </c>
+    </row>
+    <row r="835" spans="1:2" ht="78.75">
+      <c r="A835" s="2" t="s">
+        <v>1591</v>
+      </c>
+      <c r="B835" s="1" t="s">
+        <v>1592</v>
       </c>
     </row>
   </sheetData>

</xml_diff>